<commit_message>
Release Version 4.1 - Professional Ranking Engine
</commit_message>
<xml_diff>
--- a/reports/StockScanner_2026-07-13.xlsx
+++ b/reports/StockScanner_2026-07-13.xlsx
@@ -413,1078 +413,1119 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
+  <dimension ref="A1:W13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Symbol</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Market</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Current Price</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>20 MA</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>50 MA</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>200 MA</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>RSI</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>MACD</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Relative Strength</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Trend</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Entry</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Stop Loss</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Target 1</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Target 2</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Target 3</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Risk/Reward</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Suggested Shares</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Investment</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>AMD</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Semiconductor</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>538.27</v>
-      </c>
       <c r="F2" t="n">
-        <v>533.4400000000001</v>
+        <v>535.84</v>
       </c>
       <c r="G2" t="n">
-        <v>485.92</v>
+        <v>533.3200000000001</v>
       </c>
       <c r="H2" t="n">
-        <v>289.55</v>
+        <v>485.87</v>
       </c>
       <c r="I2" t="n">
-        <v>53.76</v>
+        <v>289.54</v>
       </c>
       <c r="J2" t="n">
-        <v>17.34</v>
+        <v>53.33</v>
       </c>
       <c r="K2" t="n">
-        <v>134.87</v>
+        <v>17.15</v>
       </c>
       <c r="L2" t="n">
+        <v>133.92</v>
+      </c>
+      <c r="M2" t="n">
         <v>90</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>🟢 STRONG BUY</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Strong Uptrend</t>
         </is>
       </c>
-      <c r="O2" t="n">
-        <v>533.4400000000001</v>
-      </c>
       <c r="P2" t="n">
-        <v>485.92</v>
+        <v>533.3200000000001</v>
       </c>
       <c r="Q2" t="n">
-        <v>565.45</v>
+        <v>485.87</v>
       </c>
       <c r="R2" t="n">
-        <v>586.79</v>
+        <v>565.3200000000001</v>
       </c>
       <c r="S2" t="n">
-        <v>613.46</v>
+        <v>586.66</v>
       </c>
       <c r="T2" t="n">
+        <v>613.3200000000001</v>
+      </c>
+      <c r="U2" t="n">
         <v>1.12</v>
       </c>
-      <c r="U2" t="n">
+      <c r="V2" t="n">
         <v>2</v>
       </c>
-      <c r="V2" t="n">
-        <v>1066.89</v>
+      <c r="W2" t="n">
+        <v>1066.65</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>SPY</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>ETF</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>750.34</v>
-      </c>
       <c r="F3" t="n">
-        <v>744.0599999999999</v>
+        <v>749.28</v>
       </c>
       <c r="G3" t="n">
-        <v>740.72</v>
+        <v>744</v>
       </c>
       <c r="H3" t="n">
-        <v>691.5599999999999</v>
+        <v>740.7</v>
       </c>
       <c r="I3" t="n">
-        <v>55.57</v>
+        <v>691.55</v>
       </c>
       <c r="J3" t="n">
-        <v>3.67</v>
+        <v>54.73</v>
       </c>
       <c r="K3" t="n">
+        <v>3.59</v>
+      </c>
+      <c r="L3" t="n">
         <v>0</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>90</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>🟢 STRONG BUY</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Strong Uptrend</t>
         </is>
       </c>
-      <c r="O3" t="n">
-        <v>744.0599999999999</v>
-      </c>
       <c r="P3" t="n">
-        <v>740.72</v>
+        <v>744</v>
       </c>
       <c r="Q3" t="n">
-        <v>788.7</v>
+        <v>740.7</v>
       </c>
       <c r="R3" t="n">
-        <v>818.46</v>
+        <v>788.64</v>
       </c>
       <c r="S3" t="n">
-        <v>855.66</v>
+        <v>818.4</v>
       </c>
       <c r="T3" t="n">
-        <v>22.28</v>
+        <v>855.6</v>
       </c>
       <c r="U3" t="n">
-        <v>29</v>
+        <v>22.5</v>
       </c>
       <c r="V3" t="n">
-        <v>21577.63</v>
+        <v>30</v>
+      </c>
+      <c r="W3" t="n">
+        <v>22320.1</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>PANW</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Cybersecurity</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>329.49</v>
-      </c>
       <c r="F4" t="n">
-        <v>312.79</v>
+        <v>327.4</v>
       </c>
       <c r="G4" t="n">
-        <v>270.05</v>
+        <v>312.69</v>
       </c>
       <c r="H4" t="n">
-        <v>205.37</v>
+        <v>270.01</v>
       </c>
       <c r="I4" t="n">
-        <v>59.61</v>
+        <v>205.35</v>
       </c>
       <c r="J4" t="n">
-        <v>19.72</v>
+        <v>58.98</v>
       </c>
       <c r="K4" t="n">
-        <v>63.92</v>
+        <v>19.56</v>
       </c>
       <c r="L4" t="n">
+        <v>62.96</v>
+      </c>
+      <c r="M4" t="n">
         <v>90</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>🟢 STRONG BUY</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Strong Uptrend</t>
         </is>
       </c>
-      <c r="O4" t="n">
-        <v>312.79</v>
-      </c>
       <c r="P4" t="n">
-        <v>270.05</v>
+        <v>312.69</v>
       </c>
       <c r="Q4" t="n">
-        <v>331.56</v>
+        <v>270.01</v>
       </c>
       <c r="R4" t="n">
-        <v>344.07</v>
+        <v>331.45</v>
       </c>
       <c r="S4" t="n">
-        <v>359.71</v>
+        <v>343.96</v>
       </c>
       <c r="T4" t="n">
+        <v>359.59</v>
+      </c>
+      <c r="U4" t="n">
         <v>0.73</v>
       </c>
-      <c r="U4" t="n">
+      <c r="V4" t="n">
         <v>2</v>
       </c>
-      <c r="V4" t="n">
-        <v>625.58</v>
+      <c r="W4" t="n">
+        <v>625.37</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>AMZN</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>E-Commerce</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>247.79</v>
-      </c>
       <c r="F5" t="n">
-        <v>240.51</v>
+        <v>248.4</v>
       </c>
       <c r="G5" t="n">
-        <v>253.73</v>
+        <v>240.54</v>
       </c>
       <c r="H5" t="n">
+        <v>253.74</v>
+      </c>
+      <c r="I5" t="n">
         <v>233.47</v>
       </c>
-      <c r="I5" t="n">
-        <v>53.36</v>
-      </c>
       <c r="J5" t="n">
-        <v>-1.01</v>
+        <v>53.94</v>
       </c>
       <c r="K5" t="n">
-        <v>-6.59</v>
+        <v>-0.96</v>
       </c>
       <c r="L5" t="n">
+        <v>-6.19</v>
+      </c>
+      <c r="M5" t="n">
         <v>80</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>🟢 BUY</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>253.54</v>
       </c>
-      <c r="P5" t="n">
-        <v>240.51</v>
-      </c>
       <c r="Q5" t="n">
+        <v>240.54</v>
+      </c>
+      <c r="R5" t="n">
         <v>268.75</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>278.89</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>291.57</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>1.95</v>
       </c>
-      <c r="U5" t="n">
+      <c r="V5" t="n">
         <v>7</v>
       </c>
-      <c r="V5" t="n">
+      <c r="W5" t="n">
         <v>1774.78</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>NVDA</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>204.82</v>
-      </c>
       <c r="F6" t="n">
-        <v>201.95</v>
+        <v>203.74</v>
       </c>
       <c r="G6" t="n">
-        <v>208.99</v>
+        <v>201.89</v>
       </c>
       <c r="H6" t="n">
+        <v>208.97</v>
+      </c>
+      <c r="I6" t="n">
         <v>191.6</v>
       </c>
-      <c r="I6" t="n">
-        <v>51.03</v>
-      </c>
       <c r="J6" t="n">
-        <v>-1.34</v>
+        <v>50.09</v>
       </c>
       <c r="K6" t="n">
-        <v>1.64</v>
+        <v>-1.42</v>
       </c>
       <c r="L6" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M6" t="n">
         <v>68</v>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>🟡 HOLD</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>216.13</v>
       </c>
-      <c r="P6" t="n">
-        <v>201.95</v>
-      </c>
       <c r="Q6" t="n">
+        <v>201.89</v>
+      </c>
+      <c r="R6" t="n">
         <v>229.1</v>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>237.74</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>248.55</v>
       </c>
-      <c r="T6" t="n">
+      <c r="U6" t="n">
         <v>1.52</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>7</v>
       </c>
-      <c r="V6" t="n">
+      <c r="W6" t="n">
         <v>1512.91</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="n">
+        <v>8</v>
+      </c>
+      <c r="B7" t="inlineStr">
         <is>
           <t>HOOD</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>FinTech</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>110.03</v>
-      </c>
       <c r="F7" t="n">
-        <v>105.21</v>
+        <v>109.55</v>
       </c>
       <c r="G7" t="n">
-        <v>90.33</v>
+        <v>105.19</v>
       </c>
       <c r="H7" t="n">
+        <v>90.31999999999999</v>
+      </c>
+      <c r="I7" t="n">
         <v>102.11</v>
       </c>
-      <c r="I7" t="n">
-        <v>59.08</v>
-      </c>
       <c r="J7" t="n">
-        <v>6.62</v>
+        <v>58.5</v>
       </c>
       <c r="K7" t="n">
-        <v>-17.22</v>
+        <v>6.58</v>
       </c>
       <c r="L7" t="n">
+        <v>-17.47</v>
+      </c>
+      <c r="M7" t="n">
         <v>65</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>🟡 HOLD</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>121.25</v>
       </c>
-      <c r="P7" t="n">
-        <v>105.21</v>
-      </c>
       <c r="Q7" t="n">
+        <v>105.19</v>
+      </c>
+      <c r="R7" t="n">
         <v>128.53</v>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>133.38</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>139.44</v>
       </c>
-      <c r="T7" t="n">
-        <v>0.76</v>
-      </c>
       <c r="U7" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="V7" t="n">
         <v>6</v>
       </c>
-      <c r="V7" t="n">
+      <c r="W7" t="n">
         <v>727.5</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="n">
+        <v>10</v>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>AVGO</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Semiconductor</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>388.19</v>
-      </c>
       <c r="F8" t="n">
-        <v>382.74</v>
+        <v>385.86</v>
       </c>
       <c r="G8" t="n">
-        <v>405.64</v>
+        <v>382.62</v>
       </c>
       <c r="H8" t="n">
-        <v>361.51</v>
+        <v>405.6</v>
       </c>
       <c r="I8" t="n">
-        <v>49.5</v>
+        <v>361.5</v>
       </c>
       <c r="J8" t="n">
-        <v>-4.01</v>
+        <v>48.75</v>
       </c>
       <c r="K8" t="n">
-        <v>1.15</v>
+        <v>-4.2</v>
       </c>
       <c r="L8" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="M8" t="n">
         <v>63</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>🟡 HOLD</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>418.79</v>
       </c>
-      <c r="P8" t="n">
-        <v>382.74</v>
-      </c>
       <c r="Q8" t="n">
+        <v>382.62</v>
+      </c>
+      <c r="R8" t="n">
         <v>443.91</v>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>460.67</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>481.6</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>1.16</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>2</v>
       </c>
-      <c r="V8" t="n">
+      <c r="W8" t="n">
         <v>837.5700000000001</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="n">
+        <v>3</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>META</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Internet</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>659.54</v>
-      </c>
       <c r="F9" t="n">
-        <v>589.14</v>
+        <v>662.22</v>
       </c>
       <c r="G9" t="n">
-        <v>599.91</v>
+        <v>589.27</v>
       </c>
       <c r="H9" t="n">
-        <v>641.2</v>
+        <v>599.96</v>
       </c>
       <c r="I9" t="n">
-        <v>63.57</v>
+        <v>641.22</v>
       </c>
       <c r="J9" t="n">
-        <v>12.26</v>
+        <v>64.33</v>
       </c>
       <c r="K9" t="n">
-        <v>-4.03</v>
+        <v>12.47</v>
       </c>
       <c r="L9" t="n">
+        <v>-3.46</v>
+      </c>
+      <c r="M9" t="n">
         <v>55</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>🟠 WATCH</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="O9" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>684.64</v>
       </c>
-      <c r="P9" t="n">
-        <v>589.14</v>
-      </c>
       <c r="Q9" t="n">
+        <v>589.27</v>
+      </c>
+      <c r="R9" t="n">
         <v>725.72</v>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>753.1</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>787.33</v>
       </c>
-      <c r="T9" t="n">
+      <c r="U9" t="n">
         <v>0.72</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>1</v>
       </c>
-      <c r="V9" t="n">
+      <c r="W9" t="n">
         <v>684.64</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr">
         <is>
           <t>GOOGL</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Internet</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>355.69</v>
-      </c>
       <c r="F10" t="n">
+        <v>355.7</v>
+      </c>
+      <c r="G10" t="n">
         <v>357.78</v>
       </c>
-      <c r="G10" t="n">
+      <c r="H10" t="n">
         <v>372.74</v>
       </c>
-      <c r="H10" t="n">
+      <c r="I10" t="n">
         <v>319.1</v>
       </c>
-      <c r="I10" t="n">
-        <v>45.93</v>
-      </c>
       <c r="J10" t="n">
+        <v>45.94</v>
+      </c>
+      <c r="K10" t="n">
         <v>-1.92</v>
       </c>
-      <c r="K10" t="n">
-        <v>-2.71</v>
-      </c>
       <c r="L10" t="n">
+        <v>-2.57</v>
+      </c>
+      <c r="M10" t="n">
         <v>55</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>🟠 WATCH</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>379.76</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>357.78</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>402.55</v>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>417.74</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>436.72</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>1.73</v>
       </c>
-      <c r="U10" t="n">
+      <c r="V10" t="n">
         <v>4</v>
       </c>
-      <c r="V10" t="n">
+      <c r="W10" t="n">
         <v>1519.04</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
         <is>
           <t>MSFT</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Software</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>392.76</v>
-      </c>
       <c r="F11" t="n">
-        <v>380.63</v>
+        <v>392.37</v>
       </c>
       <c r="G11" t="n">
+        <v>380.61</v>
+      </c>
+      <c r="H11" t="n">
         <v>402.71</v>
       </c>
-      <c r="H11" t="n">
+      <c r="I11" t="n">
         <v>440.14</v>
       </c>
-      <c r="I11" t="n">
-        <v>51.95</v>
-      </c>
       <c r="J11" t="n">
-        <v>-4.33</v>
+        <v>51.75</v>
       </c>
       <c r="K11" t="n">
-        <v>-24.9</v>
+        <v>-4.36</v>
       </c>
       <c r="L11" t="n">
+        <v>-24.85</v>
+      </c>
+      <c r="M11" t="n">
         <v>35</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>🔴 AVOID</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
+      <c r="O11" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>405.77</v>
       </c>
-      <c r="P11" t="n">
-        <v>380.63</v>
-      </c>
       <c r="Q11" t="n">
+        <v>380.61</v>
+      </c>
+      <c r="R11" t="n">
         <v>430.11</v>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>446.34</v>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>466.63</v>
       </c>
-      <c r="T11" t="n">
+      <c r="U11" t="n">
         <v>1.61</v>
       </c>
-      <c r="U11" t="n">
+      <c r="V11" t="n">
         <v>3</v>
       </c>
-      <c r="V11" t="n">
+      <c r="W11" t="n">
         <v>1217.3</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>PLTR</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>AI</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>130.14</v>
-      </c>
       <c r="F12" t="n">
-        <v>124.87</v>
+        <v>129.27</v>
       </c>
       <c r="G12" t="n">
-        <v>133.1</v>
+        <v>124.83</v>
       </c>
       <c r="H12" t="n">
+        <v>133.08</v>
+      </c>
+      <c r="I12" t="n">
         <v>156.54</v>
       </c>
-      <c r="I12" t="n">
-        <v>51.52</v>
-      </c>
       <c r="J12" t="n">
-        <v>-1.09</v>
+        <v>50.68</v>
       </c>
       <c r="K12" t="n">
-        <v>-36</v>
+        <v>-1.16</v>
       </c>
       <c r="L12" t="n">
+        <v>-36.35</v>
+      </c>
+      <c r="M12" t="n">
         <v>35</v>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>🔴 AVOID</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
+      <c r="O12" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="O12" t="n">
+      <c r="P12" t="n">
         <v>140.29</v>
       </c>
-      <c r="P12" t="n">
-        <v>124.87</v>
-      </c>
       <c r="Q12" t="n">
+        <v>124.83</v>
+      </c>
+      <c r="R12" t="n">
         <v>148.71</v>
       </c>
-      <c r="R12" t="n">
+      <c r="S12" t="n">
         <v>154.32</v>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>161.33</v>
       </c>
-      <c r="T12" t="n">
+      <c r="U12" t="n">
         <v>0.91</v>
       </c>
-      <c r="U12" t="n">
+      <c r="V12" t="n">
         <v>6</v>
       </c>
-      <c r="V12" t="n">
+      <c r="W12" t="n">
         <v>841.73</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
         <is>
           <t>TSLA</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>NASDAQ</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>EV</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>393.9</v>
-      </c>
       <c r="F13" t="n">
-        <v>400.61</v>
+        <v>392.76</v>
       </c>
       <c r="G13" t="n">
-        <v>409.62</v>
+        <v>400.56</v>
       </c>
       <c r="H13" t="n">
-        <v>417.98</v>
+        <v>409.6</v>
       </c>
       <c r="I13" t="n">
-        <v>46.97</v>
+        <v>417.97</v>
       </c>
       <c r="J13" t="n">
-        <v>-0.93</v>
+        <v>46.66</v>
       </c>
       <c r="K13" t="n">
-        <v>-20.64</v>
+        <v>-1.02</v>
       </c>
       <c r="L13" t="n">
+        <v>-20.75</v>
+      </c>
+      <c r="M13" t="n">
         <v>10</v>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>🔴 AVOID</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
+      <c r="O13" t="inlineStr">
         <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="O13" t="n">
+      <c r="P13" t="n">
         <v>437.19</v>
       </c>
-      <c r="P13" t="n">
-        <v>400.61</v>
-      </c>
       <c r="Q13" t="n">
+        <v>400.56</v>
+      </c>
+      <c r="R13" t="n">
         <v>463.42</v>
       </c>
-      <c r="R13" t="n">
+      <c r="S13" t="n">
         <v>480.91</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>502.77</v>
       </c>
-      <c r="T13" t="n">
-        <v>1.2</v>
-      </c>
       <c r="U13" t="n">
+        <v>1.19</v>
+      </c>
+      <c r="V13" t="n">
         <v>2</v>
       </c>
-      <c r="V13" t="n">
+      <c r="W13" t="n">
         <v>874.38</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Release Version 4.2 - AI Buy Signal Engine
</commit_message>
<xml_diff>
--- a/reports/StockScanner_2026-07-13.xlsx
+++ b/reports/StockScanner_2026-07-13.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W13"/>
+  <dimension ref="A1:X13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -489,45 +489,50 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
           <t>Trend</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Entry</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Stop Loss</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Target 1</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Target 2</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Target 3</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Risk/Reward</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Suggested Shares</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Investment</t>
         </is>
@@ -558,25 +563,25 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>535.84</v>
+        <v>535.01</v>
       </c>
       <c r="G2" t="n">
-        <v>533.3200000000001</v>
+        <v>533.28</v>
       </c>
       <c r="H2" t="n">
-        <v>485.87</v>
+        <v>485.85</v>
       </c>
       <c r="I2" t="n">
-        <v>289.54</v>
+        <v>289.53</v>
       </c>
       <c r="J2" t="n">
-        <v>53.33</v>
+        <v>53.19</v>
       </c>
       <c r="K2" t="n">
-        <v>17.15</v>
+        <v>17.08</v>
       </c>
       <c r="L2" t="n">
-        <v>133.92</v>
+        <v>133.63</v>
       </c>
       <c r="M2" t="n">
         <v>90</v>
@@ -588,32 +593,37 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>🟢 Pullback to 20 MA</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>Strong Uptrend</t>
         </is>
       </c>
-      <c r="P2" t="n">
-        <v>533.3200000000001</v>
-      </c>
       <c r="Q2" t="n">
-        <v>485.87</v>
+        <v>533.28</v>
       </c>
       <c r="R2" t="n">
-        <v>565.3200000000001</v>
+        <v>485.85</v>
       </c>
       <c r="S2" t="n">
-        <v>586.66</v>
+        <v>565.28</v>
       </c>
       <c r="T2" t="n">
-        <v>613.3200000000001</v>
+        <v>586.61</v>
       </c>
       <c r="U2" t="n">
+        <v>613.27</v>
+      </c>
+      <c r="V2" t="n">
         <v>1.12</v>
       </c>
-      <c r="V2" t="n">
-        <v>2</v>
-      </c>
       <c r="W2" t="n">
-        <v>1066.65</v>
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -641,22 +651,22 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>749.28</v>
+        <v>748.63</v>
       </c>
       <c r="G3" t="n">
-        <v>744</v>
+        <v>743.97</v>
       </c>
       <c r="H3" t="n">
-        <v>740.7</v>
+        <v>740.6799999999999</v>
       </c>
       <c r="I3" t="n">
         <v>691.55</v>
       </c>
       <c r="J3" t="n">
-        <v>54.73</v>
+        <v>54.23</v>
       </c>
       <c r="K3" t="n">
-        <v>3.59</v>
+        <v>3.54</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -671,32 +681,37 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>🟢 Strong Uptrend</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
           <t>Strong Uptrend</t>
         </is>
       </c>
-      <c r="P3" t="n">
-        <v>744</v>
-      </c>
       <c r="Q3" t="n">
-        <v>740.7</v>
+        <v>743.97</v>
       </c>
       <c r="R3" t="n">
-        <v>788.64</v>
+        <v>740.6799999999999</v>
       </c>
       <c r="S3" t="n">
-        <v>818.4</v>
+        <v>788.61</v>
       </c>
       <c r="T3" t="n">
-        <v>855.6</v>
+        <v>818.37</v>
       </c>
       <c r="U3" t="n">
-        <v>22.5</v>
+        <v>855.5700000000001</v>
       </c>
       <c r="V3" t="n">
-        <v>30</v>
+        <v>22.63</v>
       </c>
       <c r="W3" t="n">
-        <v>22320.1</v>
+        <v>3</v>
+      </c>
+      <c r="X3" t="n">
+        <v>2231.91</v>
       </c>
     </row>
     <row r="4">
@@ -724,25 +739,25 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>327.4</v>
+        <v>326.65</v>
       </c>
       <c r="G4" t="n">
-        <v>312.69</v>
+        <v>312.65</v>
       </c>
       <c r="H4" t="n">
-        <v>270.01</v>
+        <v>269.99</v>
       </c>
       <c r="I4" t="n">
         <v>205.35</v>
       </c>
       <c r="J4" t="n">
-        <v>58.98</v>
+        <v>58.75</v>
       </c>
       <c r="K4" t="n">
-        <v>19.56</v>
+        <v>19.5</v>
       </c>
       <c r="L4" t="n">
-        <v>62.96</v>
+        <v>62.67</v>
       </c>
       <c r="M4" t="n">
         <v>90</v>
@@ -754,32 +769,37 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>⚪ Neutral</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>Strong Uptrend</t>
         </is>
       </c>
-      <c r="P4" t="n">
-        <v>312.69</v>
-      </c>
       <c r="Q4" t="n">
-        <v>270.01</v>
+        <v>312.65</v>
       </c>
       <c r="R4" t="n">
-        <v>331.45</v>
+        <v>269.99</v>
       </c>
       <c r="S4" t="n">
-        <v>343.96</v>
+        <v>331.41</v>
       </c>
       <c r="T4" t="n">
-        <v>359.59</v>
+        <v>343.91</v>
       </c>
       <c r="U4" t="n">
+        <v>359.55</v>
+      </c>
+      <c r="V4" t="n">
         <v>0.73</v>
       </c>
-      <c r="V4" t="n">
-        <v>2</v>
-      </c>
       <c r="W4" t="n">
-        <v>625.37</v>
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -807,25 +827,25 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>248.4</v>
+        <v>246.9</v>
       </c>
       <c r="G5" t="n">
-        <v>240.54</v>
+        <v>240.46</v>
       </c>
       <c r="H5" t="n">
-        <v>253.74</v>
+        <v>253.71</v>
       </c>
       <c r="I5" t="n">
-        <v>233.47</v>
+        <v>233.46</v>
       </c>
       <c r="J5" t="n">
-        <v>53.94</v>
+        <v>52.51</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.96</v>
+        <v>-1.08</v>
       </c>
       <c r="L5" t="n">
-        <v>-6.19</v>
+        <v>-6.72</v>
       </c>
       <c r="M5" t="n">
         <v>80</v>
@@ -837,32 +857,37 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
+          <t>⚪ Neutral</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>253.54</v>
       </c>
-      <c r="Q5" t="n">
-        <v>240.54</v>
-      </c>
       <c r="R5" t="n">
+        <v>240.46</v>
+      </c>
+      <c r="S5" t="n">
         <v>268.75</v>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>278.89</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>291.57</v>
       </c>
-      <c r="U5" t="n">
-        <v>1.95</v>
-      </c>
       <c r="V5" t="n">
-        <v>7</v>
+        <v>1.94</v>
       </c>
       <c r="W5" t="n">
-        <v>1774.78</v>
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -890,10 +915,10 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>203.74</v>
+        <v>203.76</v>
       </c>
       <c r="G6" t="n">
-        <v>201.89</v>
+        <v>201.9</v>
       </c>
       <c r="H6" t="n">
         <v>208.97</v>
@@ -902,13 +927,13 @@
         <v>191.6</v>
       </c>
       <c r="J6" t="n">
-        <v>50.09</v>
+        <v>50.12</v>
       </c>
       <c r="K6" t="n">
         <v>-1.42</v>
       </c>
       <c r="L6" t="n">
-        <v>1.2</v>
+        <v>1.32</v>
       </c>
       <c r="M6" t="n">
         <v>68</v>
@@ -920,32 +945,37 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>⚪ Neutral</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>216.13</v>
       </c>
-      <c r="Q6" t="n">
-        <v>201.89</v>
-      </c>
       <c r="R6" t="n">
+        <v>201.9</v>
+      </c>
+      <c r="S6" t="n">
         <v>229.1</v>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>237.74</v>
       </c>
-      <c r="T6" t="n">
+      <c r="U6" t="n">
         <v>248.55</v>
       </c>
-      <c r="U6" t="n">
+      <c r="V6" t="n">
         <v>1.52</v>
       </c>
-      <c r="V6" t="n">
-        <v>7</v>
-      </c>
       <c r="W6" t="n">
-        <v>1512.91</v>
+        <v>0</v>
+      </c>
+      <c r="X6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -973,10 +1003,10 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>109.55</v>
+        <v>109.36</v>
       </c>
       <c r="G7" t="n">
-        <v>105.19</v>
+        <v>105.18</v>
       </c>
       <c r="H7" t="n">
         <v>90.31999999999999</v>
@@ -985,13 +1015,13 @@
         <v>102.11</v>
       </c>
       <c r="J7" t="n">
-        <v>58.5</v>
+        <v>58.28</v>
       </c>
       <c r="K7" t="n">
-        <v>6.58</v>
+        <v>6.57</v>
       </c>
       <c r="L7" t="n">
-        <v>-17.47</v>
+        <v>-17.53</v>
       </c>
       <c r="M7" t="n">
         <v>65</v>
@@ -1003,32 +1033,37 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
+          <t>⚪ Neutral</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>121.25</v>
       </c>
-      <c r="Q7" t="n">
-        <v>105.19</v>
-      </c>
       <c r="R7" t="n">
+        <v>105.18</v>
+      </c>
+      <c r="S7" t="n">
         <v>128.53</v>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>133.38</v>
       </c>
-      <c r="T7" t="n">
+      <c r="U7" t="n">
         <v>139.44</v>
       </c>
-      <c r="U7" t="n">
+      <c r="V7" t="n">
         <v>0.75</v>
       </c>
-      <c r="V7" t="n">
-        <v>6</v>
-      </c>
       <c r="W7" t="n">
-        <v>727.5</v>
+        <v>0</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -1056,25 +1091,25 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>385.86</v>
+        <v>385.44</v>
       </c>
       <c r="G8" t="n">
-        <v>382.62</v>
+        <v>382.6</v>
       </c>
       <c r="H8" t="n">
-        <v>405.6</v>
+        <v>405.59</v>
       </c>
       <c r="I8" t="n">
         <v>361.5</v>
       </c>
       <c r="J8" t="n">
-        <v>48.75</v>
+        <v>48.61</v>
       </c>
       <c r="K8" t="n">
-        <v>-4.2</v>
+        <v>-4.23</v>
       </c>
       <c r="L8" t="n">
-        <v>0.64</v>
+        <v>0.61</v>
       </c>
       <c r="M8" t="n">
         <v>63</v>
@@ -1086,32 +1121,37 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
+          <t>⚪ Neutral</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>418.79</v>
       </c>
-      <c r="Q8" t="n">
-        <v>382.62</v>
-      </c>
       <c r="R8" t="n">
+        <v>382.6</v>
+      </c>
+      <c r="S8" t="n">
         <v>443.91</v>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>460.67</v>
       </c>
-      <c r="T8" t="n">
+      <c r="U8" t="n">
         <v>481.6</v>
       </c>
-      <c r="U8" t="n">
+      <c r="V8" t="n">
         <v>1.16</v>
       </c>
-      <c r="V8" t="n">
-        <v>2</v>
-      </c>
       <c r="W8" t="n">
-        <v>837.5700000000001</v>
+        <v>0</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -1139,25 +1179,25 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>662.22</v>
+        <v>657.45</v>
       </c>
       <c r="G9" t="n">
-        <v>589.27</v>
+        <v>589.03</v>
       </c>
       <c r="H9" t="n">
-        <v>599.96</v>
+        <v>599.86</v>
       </c>
       <c r="I9" t="n">
-        <v>641.22</v>
+        <v>641.1900000000001</v>
       </c>
       <c r="J9" t="n">
-        <v>64.33</v>
+        <v>63</v>
       </c>
       <c r="K9" t="n">
-        <v>12.47</v>
+        <v>12.09</v>
       </c>
       <c r="L9" t="n">
-        <v>-3.46</v>
+        <v>-4.14</v>
       </c>
       <c r="M9" t="n">
         <v>55</v>
@@ -1169,32 +1209,37 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
+          <t>⚪ Neutral</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>684.64</v>
       </c>
-      <c r="Q9" t="n">
-        <v>589.27</v>
-      </c>
       <c r="R9" t="n">
+        <v>589.03</v>
+      </c>
+      <c r="S9" t="n">
         <v>725.72</v>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>753.1</v>
       </c>
-      <c r="T9" t="n">
+      <c r="U9" t="n">
         <v>787.33</v>
       </c>
-      <c r="U9" t="n">
+      <c r="V9" t="n">
         <v>0.72</v>
       </c>
-      <c r="V9" t="n">
-        <v>1</v>
-      </c>
       <c r="W9" t="n">
-        <v>684.64</v>
+        <v>0</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -1222,25 +1267,25 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>355.7</v>
+        <v>353.02</v>
       </c>
       <c r="G10" t="n">
-        <v>357.78</v>
+        <v>357.65</v>
       </c>
       <c r="H10" t="n">
-        <v>372.74</v>
+        <v>372.69</v>
       </c>
       <c r="I10" t="n">
-        <v>319.1</v>
+        <v>319.09</v>
       </c>
       <c r="J10" t="n">
-        <v>45.94</v>
+        <v>44.12</v>
       </c>
       <c r="K10" t="n">
-        <v>-1.92</v>
+        <v>-2.13</v>
       </c>
       <c r="L10" t="n">
-        <v>-2.57</v>
+        <v>-3.28</v>
       </c>
       <c r="M10" t="n">
         <v>55</v>
@@ -1252,41 +1297,46 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
+          <t>⚪ Neutral</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>379.76</v>
       </c>
-      <c r="Q10" t="n">
-        <v>357.78</v>
-      </c>
       <c r="R10" t="n">
+        <v>357.65</v>
+      </c>
+      <c r="S10" t="n">
         <v>402.55</v>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>417.74</v>
       </c>
-      <c r="T10" t="n">
+      <c r="U10" t="n">
         <v>436.72</v>
       </c>
-      <c r="U10" t="n">
-        <v>1.73</v>
-      </c>
       <c r="V10" t="n">
-        <v>4</v>
+        <v>1.72</v>
       </c>
       <c r="W10" t="n">
-        <v>1519.04</v>
+        <v>0</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>PLTR</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1296,34 +1346,34 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Software</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>392.37</v>
+        <v>128.71</v>
       </c>
       <c r="G11" t="n">
-        <v>380.61</v>
+        <v>124.8</v>
       </c>
       <c r="H11" t="n">
-        <v>402.71</v>
+        <v>133.07</v>
       </c>
       <c r="I11" t="n">
-        <v>440.14</v>
+        <v>156.53</v>
       </c>
       <c r="J11" t="n">
-        <v>51.75</v>
+        <v>50.12</v>
       </c>
       <c r="K11" t="n">
-        <v>-4.36</v>
+        <v>-1.2</v>
       </c>
       <c r="L11" t="n">
-        <v>-24.85</v>
+        <v>-36.58</v>
       </c>
       <c r="M11" t="n">
         <v>35</v>
@@ -1335,41 +1385,46 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
+          <t>⚪ Neutral</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="P11" t="n">
-        <v>405.77</v>
-      </c>
       <c r="Q11" t="n">
-        <v>380.61</v>
+        <v>140.29</v>
       </c>
       <c r="R11" t="n">
-        <v>430.11</v>
+        <v>124.8</v>
       </c>
       <c r="S11" t="n">
-        <v>446.34</v>
+        <v>148.71</v>
       </c>
       <c r="T11" t="n">
-        <v>466.63</v>
+        <v>154.32</v>
       </c>
       <c r="U11" t="n">
-        <v>1.61</v>
+        <v>161.33</v>
       </c>
       <c r="V11" t="n">
-        <v>3</v>
+        <v>0.91</v>
       </c>
       <c r="W11" t="n">
-        <v>1217.3</v>
+        <v>0</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PLTR</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1379,37 +1434,37 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>AI</t>
+          <t>Software</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>129.27</v>
+        <v>390.66</v>
       </c>
       <c r="G12" t="n">
-        <v>124.83</v>
+        <v>380.53</v>
       </c>
       <c r="H12" t="n">
-        <v>133.08</v>
+        <v>402.67</v>
       </c>
       <c r="I12" t="n">
-        <v>156.54</v>
+        <v>440.13</v>
       </c>
       <c r="J12" t="n">
-        <v>50.68</v>
+        <v>50.82</v>
       </c>
       <c r="K12" t="n">
-        <v>-1.16</v>
+        <v>-4.49</v>
       </c>
       <c r="L12" t="n">
-        <v>-36.35</v>
+        <v>-25.12</v>
       </c>
       <c r="M12" t="n">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -1418,32 +1473,37 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
+          <t>⚪ Neutral</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="P12" t="n">
-        <v>140.29</v>
-      </c>
       <c r="Q12" t="n">
-        <v>124.83</v>
+        <v>405.77</v>
       </c>
       <c r="R12" t="n">
-        <v>148.71</v>
+        <v>380.53</v>
       </c>
       <c r="S12" t="n">
-        <v>154.32</v>
+        <v>430.11</v>
       </c>
       <c r="T12" t="n">
-        <v>161.33</v>
+        <v>446.34</v>
       </c>
       <c r="U12" t="n">
-        <v>0.91</v>
+        <v>466.63</v>
       </c>
       <c r="V12" t="n">
-        <v>6</v>
+        <v>1.61</v>
       </c>
       <c r="W12" t="n">
-        <v>841.73</v>
+        <v>0</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="13">
@@ -1471,25 +1531,25 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>392.76</v>
+        <v>392.51</v>
       </c>
       <c r="G13" t="n">
-        <v>400.56</v>
+        <v>400.54</v>
       </c>
       <c r="H13" t="n">
-        <v>409.6</v>
+        <v>409.59</v>
       </c>
       <c r="I13" t="n">
         <v>417.97</v>
       </c>
       <c r="J13" t="n">
-        <v>46.66</v>
+        <v>46.59</v>
       </c>
       <c r="K13" t="n">
-        <v>-1.02</v>
+        <v>-1.04</v>
       </c>
       <c r="L13" t="n">
-        <v>-20.75</v>
+        <v>-20.72</v>
       </c>
       <c r="M13" t="n">
         <v>10</v>
@@ -1501,32 +1561,37 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
+          <t>⚪ Neutral</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
           <t>Breakout</t>
         </is>
       </c>
-      <c r="P13" t="n">
+      <c r="Q13" t="n">
         <v>437.19</v>
       </c>
-      <c r="Q13" t="n">
-        <v>400.56</v>
-      </c>
       <c r="R13" t="n">
+        <v>400.54</v>
+      </c>
+      <c r="S13" t="n">
         <v>463.42</v>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>480.91</v>
       </c>
-      <c r="T13" t="n">
+      <c r="U13" t="n">
         <v>502.77</v>
       </c>
-      <c r="U13" t="n">
+      <c r="V13" t="n">
         <v>1.19</v>
       </c>
-      <c r="V13" t="n">
-        <v>2</v>
-      </c>
       <c r="W13" t="n">
-        <v>874.38</v>
+        <v>0</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>